<commit_message>
0.5.1 new sprite soldier
</commit_message>
<xml_diff>
--- a/Armi.xlsx
+++ b/Armi.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source Code\no-mans-ground\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3CA2164-8394-453E-86C1-A859FCCA9ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FCB17C-AD7F-49C6-B916-880CD41A414B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{F76167B4-6CF2-454C-82A2-0FD2AAE3E619}"/>
   </bookViews>
   <sheets>
     <sheet name="Esercito" sheetId="1" r:id="rId1"/>
-    <sheet name="Foglio2" sheetId="2" r:id="rId2"/>
+    <sheet name="Armi" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Esercito</t>
   </si>
@@ -110,21 +110,143 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Precisione</t>
-  </si>
-  <si>
-    <t>Danni</t>
-  </si>
-  <si>
     <t>Aggiunta fatica</t>
+  </si>
+  <si>
+    <t>Precisione (0-20)</t>
+  </si>
+  <si>
+    <t>Danni (0-100)</t>
+  </si>
+  <si>
+    <t>Colore</t>
+  </si>
+  <si>
+    <t>Codice HEX</t>
+  </si>
+  <si>
+    <t>#4D5D53</t>
+  </si>
+  <si>
+    <r>
+      <t>Feldgrau</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Grigio campo)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hechtgrau</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Grigio luccio) </t>
+    </r>
+  </si>
+  <si>
+    <t>#75838F</t>
+  </si>
+  <si>
+    <r>
+      <t>Bleu Horizon</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Blu orizzonte)</t>
+    </r>
+  </si>
+  <si>
+    <t>#7CA2B8</t>
+  </si>
+  <si>
+    <r>
+      <t>Khaki</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Cachi britannico)</t>
+    </r>
+  </si>
+  <si>
+    <t>#625D43</t>
+  </si>
+  <si>
+    <r>
+      <t>Zashchitny</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Verde protettivo / Oliva russo)</t>
+    </r>
+  </si>
+  <si>
+    <t>#525838</t>
+  </si>
+  <si>
+    <r>
+      <t>Grigio-Verde</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>#5F6C37</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -152,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -160,6 +282,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -494,45 +617,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9138AD7C-5B9A-4FFA-8442-D181E819F221}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
+      <c r="B6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>1</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -583,13 +750,13 @@
         <v>18</v>
       </c>
       <c r="J1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" t="s">
         <v>21</v>
-      </c>
-      <c r="K1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="331.2" x14ac:dyDescent="0.3">
@@ -619,6 +786,15 @@
       </c>
       <c r="I2" s="1" t="s">
         <v>19</v>
+      </c>
+      <c r="J2">
+        <v>14</v>
+      </c>
+      <c r="K2">
+        <v>20</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
0.5.4 Armi e munizioni
</commit_message>
<xml_diff>
--- a/Armi.xlsx
+++ b/Armi.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source Code\no-mans-ground\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Source Code\no-mans-ground\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FCB17C-AD7F-49C6-B916-880CD41A414B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F421E3C-981C-4206-9157-6A08D1589F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{F76167B4-6CF2-454C-82A2-0FD2AAE3E619}"/>
+    <workbookView xWindow="16470" yWindow="4440" windowWidth="33780" windowHeight="16440" xr2:uid="{F76167B4-6CF2-454C-82A2-0FD2AAE3E619}"/>
   </bookViews>
   <sheets>
     <sheet name="Esercito" sheetId="1" r:id="rId1"/>
-    <sheet name="Armi" sheetId="2" r:id="rId2"/>
+    <sheet name="Tipo Armi" sheetId="3" r:id="rId2"/>
+    <sheet name="Armi" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
   <si>
     <t>Esercito</t>
   </si>
@@ -231,6 +232,27 @@
   </si>
   <si>
     <t>#5F6C37</t>
+  </si>
+  <si>
+    <t>Arma default</t>
+  </si>
+  <si>
+    <t>Pistola</t>
+  </si>
+  <si>
+    <t>Mitragliatrice Leggere</t>
+  </si>
+  <si>
+    <t>Mitragliatrice Pesante</t>
+  </si>
+  <si>
+    <t>Bombe a mano</t>
+  </si>
+  <si>
+    <t>Artiglieria</t>
+  </si>
+  <si>
+    <t>Arma Bianca</t>
   </si>
 </sst>
 </file>
@@ -617,111 +639,186 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9138AD7C-5B9A-4FFA-8442-D181E819F221}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C30E1343-9FE3-4520-9977-BD87B86F76F9}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F96968F-DB13-4923-AB82-189DC5028C3F}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="60" customWidth="1"/>
-    <col min="8" max="8" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -759,7 +856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="331.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="360" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>

</xml_diff>